<commit_message>
Update example_fields.xlsx with new data: revised content to enhance indexing capabilities and improve overall data quality.
</commit_message>
<xml_diff>
--- a/knowledge_base/files/example_fields.xlsx
+++ b/knowledge_base/files/example_fields.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t xml:space="preserve">水果</t>
   </si>
@@ -44,12 +44,6 @@
   </si>
   <si>
     <t xml:space="preserve">魚肉</t>
-  </si>
-  <si>
-    <t xml:space="preserve">火龍果</t>
-  </si>
-  <si>
-    <t xml:space="preserve">鴕鳥肉</t>
   </si>
 </sst>
 </file>
@@ -330,7 +324,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -363,14 +357,6 @@
       </c>
       <c r="B4" s="1" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="0" t="s">
-        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>